<commit_message>
il ilce sistemi eklendi
</commit_message>
<xml_diff>
--- a/paragraf_koçu_kazanım_çeşitleri.xlsx
+++ b/paragraf_koçu_kazanım_çeşitleri.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahmet/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahmet/Documents/projeler/yayindenizi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3993C597-10F1-D74A-ACD2-F591E0FD5DE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B50507C-B055-0F4A-A7EC-8EADD990C3F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5820" yWindow="2540" windowWidth="25960" windowHeight="16240" xr2:uid="{0AD648B7-BCA6-CC44-9C04-DD3BB970AB0E}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{0AD648B7-BCA6-CC44-9C04-DD3BB970AB0E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>Paragrafın Yorumlanması</t>
   </si>
@@ -68,22 +68,6 @@
     <t>21.3</t>
   </si>
   <si>
-    <t>Bir Paragrafa Bağlı Çoklu Sorular
-Paragrafta Yardımcı Düşünceler</t>
-  </si>
-  <si>
-    <t>21.5.11
-21.5.2</t>
-  </si>
-  <si>
-    <t>Bir Paragrafa Bağlı Çoklu Sorular
-Paragrafın Konusu</t>
-  </si>
-  <si>
-    <t>21.5.11
-21.5.6</t>
-  </si>
-  <si>
     <t>Paragrafta Ana Düşünce (Ana Fikir)</t>
   </si>
   <si>
@@ -126,50 +110,16 @@
     <t>21.4.5</t>
   </si>
   <si>
-    <t>Bir Paragrafa Bağlı Çoklu Sorular
-Paragrafta Ana Düşünce (Ana Fikir)</t>
-  </si>
-  <si>
-    <t>21.5.11
-21.5.1</t>
-  </si>
-  <si>
-    <t>Bir Paragrafa Bağlı Çoklu Sorular
-Paragrafta Boş Bırakılan Yerleri Tamamlama</t>
-  </si>
-  <si>
-    <t>21.5.11
-21.4.2</t>
-  </si>
-  <si>
-    <t>Bir Paragrafa Bağlı Çoklu Sorular
-ANLATIM TEKNİKLERİ VE DÜŞÜNCEYİ GELİŞTİRME YOLLARI</t>
-  </si>
-  <si>
-    <t>21.5.11
-21.3</t>
-  </si>
-  <si>
-    <t>Bir Paragrafa Bağlı Çoklu Sorular
-Paragrafın Karşılık Olduğu Soruyu Belirleme</t>
-  </si>
-  <si>
-    <t>21.5.11
-21.5.3</t>
-  </si>
-  <si>
     <t>Paragrafa Özgü Soru Kökü</t>
   </si>
   <si>
     <t>21.5.10</t>
   </si>
   <si>
-    <t>Bir Paragrafa Bağlı Çoklu Sorular
-Paragrafın Yorumlanması</t>
-  </si>
-  <si>
-    <t>21.5.11
-21.5.4</t>
+    <t>21.5.11</t>
+  </si>
+  <si>
+    <t>Bir Paragrafa Bağlı Çoklu Sorular</t>
   </si>
 </sst>
 </file>
@@ -583,10 +533,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78500645-5593-0D48-A5E8-CD9F79FD6E36}">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="49.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
@@ -630,18 +581,18 @@
       </c>
     </row>
     <row r="6" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>13</v>
       </c>
     </row>
@@ -694,62 +645,19 @@
       </c>
     </row>
     <row r="14" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
+    </row>
+    <row r="15" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="16" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="17" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="18" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>